<commit_message>
Update Primary template subjects to match academic-performance CSV
</commit_message>
<xml_diff>
--- a/Hiktaos_Primary_Final.xlsx
+++ b/Hiktaos_Primary_Final.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="145">
   <si>
     <t>HIKTAOS</t>
   </si>
@@ -116,9 +116,6 @@
     <t>Attendance Percentage</t>
   </si>
   <si>
-    <t>%</t>
-  </si>
-  <si>
     <t>ACADEMIC PERFORMANCE</t>
   </si>
   <si>
@@ -153,49 +150,52 @@
 IN SUBJECT</t>
   </si>
   <si>
-    <t>English Studies</t>
+    <t>Social Studies</t>
+  </si>
+  <si>
+    <t>Civic Education</t>
+  </si>
+  <si>
+    <t>CRS</t>
+  </si>
+  <si>
+    <t>Security Education</t>
+  </si>
+  <si>
+    <t>History</t>
+  </si>
+  <si>
+    <t>Agricultural Science</t>
+  </si>
+  <si>
+    <t>Home Economics</t>
+  </si>
+  <si>
+    <t>Basic Science</t>
+  </si>
+  <si>
+    <t>PHE</t>
+  </si>
+  <si>
+    <t>ICT</t>
+  </si>
+  <si>
+    <t>Cultural &amp; Creative Arts</t>
   </si>
   <si>
     <t>Mathematics</t>
   </si>
   <si>
-    <t>Basic Science &amp; Tech</t>
-  </si>
-  <si>
-    <t>Social Studies</t>
-  </si>
-  <si>
-    <t>Civic Education</t>
-  </si>
-  <si>
-    <t>Cultural &amp; Creative Arts</t>
-  </si>
-  <si>
-    <t>Physical &amp; Health Education</t>
-  </si>
-  <si>
-    <t>Agricultural Science</t>
-  </si>
-  <si>
-    <t>Home Economics</t>
-  </si>
-  <si>
-    <t>CRS / IRS</t>
-  </si>
-  <si>
-    <t>Yoruba Language</t>
+    <t>English Language</t>
+  </si>
+  <si>
+    <t>Verbal Reasoning</t>
   </si>
   <si>
     <t>Quantitative Reasoning</t>
   </si>
   <si>
-    <t>Verbal Reasoning</t>
-  </si>
-  <si>
-    <t>Handwriting</t>
-  </si>
-  <si>
-    <t>French</t>
+    <t>Vocational Studies</t>
   </si>
   <si>
     <t>TOTAL MARKS</t>
@@ -759,8 +759,8 @@
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>136398</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>12573</xdr:rowOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>136398</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1081,7 +1081,7 @@
     <col min="1" max="26" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="40" customHeight="1">
+    <row r="1" spans="1:26">
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1446,9 +1446,7 @@
       <c r="J17" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="M17" s="13" t="s">
-        <v>9</v>
-      </c>
+      <c r="M17" s="14"/>
       <c r="N17" s="14"/>
       <c r="O17" s="14"/>
       <c r="P17" s="14"/>
@@ -1550,9 +1548,6 @@
       <c r="W20" s="13"/>
       <c r="X20" s="15"/>
       <c r="Y20" s="15"/>
-      <c r="Z20" s="13" t="s">
-        <v>33</v>
-      </c>
     </row>
     <row r="21" spans="1:26">
       <c r="A21" s="13" t="s">
@@ -1607,7 +1602,7 @@
     </row>
     <row r="24" spans="1:26">
       <c r="A24" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -1638,34 +1633,34 @@
     </row>
     <row r="25" spans="1:26">
       <c r="A25" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="B25" s="16" t="s">
-        <v>36</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
       <c r="G25" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K25" s="16"/>
       <c r="L25" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="M25" s="16"/>
       <c r="N25" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O25" s="16"/>
       <c r="P25" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q25" s="16"/>
       <c r="R25" s="16"/>
@@ -1673,7 +1668,7 @@
         <v>68</v>
       </c>
       <c r="U25" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="V25" s="17"/>
       <c r="W25" s="17" t="s">
@@ -1691,10 +1686,10 @@
       <c r="E26" s="16"/>
       <c r="F26" s="16"/>
       <c r="G26" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H26" s="16" t="s">
         <v>38</v>
-      </c>
-      <c r="H26" s="16" t="s">
-        <v>39</v>
       </c>
       <c r="I26" s="16"/>
       <c r="J26" s="16"/>
@@ -1727,7 +1722,7 @@
         <v>1</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="19"/>
@@ -1744,7 +1739,7 @@
       </c>
       <c r="M28" s="18"/>
       <c r="N28" s="18">
-        <f>IF(L28&gt;=75,"A1",IF(L28&gt;=70,"B2",IF(L28&gt;=65,"B3",IF(L28&gt;=60,"C4",IF(L28&gt;=55,"C5",IF(L28&gt;=50,"C6",IF(N28&gt;=45,"D7",IF(L28&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L28&gt;=75,"A1",IF(L28&gt;=70,"B2",IF(L28&gt;=65,"B3",IF(L28&gt;=60,"C4",IF(L28&gt;=55,"C5",IF(L28&gt;=50,"C6",IF(L28&gt;=45,"D7",IF(L28&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O28" s="18"/>
@@ -1770,7 +1765,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="19"/>
@@ -1787,7 +1782,7 @@
       </c>
       <c r="M29" s="18"/>
       <c r="N29" s="18">
-        <f>IF(L29&gt;=75,"A1",IF(L29&gt;=70,"B2",IF(L29&gt;=65,"B3",IF(L29&gt;=60,"C4",IF(L29&gt;=55,"C5",IF(L29&gt;=50,"C6",IF(N29&gt;=45,"D7",IF(L29&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L29&gt;=75,"A1",IF(L29&gt;=70,"B2",IF(L29&gt;=65,"B3",IF(L29&gt;=60,"C4",IF(L29&gt;=55,"C5",IF(L29&gt;=50,"C6",IF(L29&gt;=45,"D7",IF(L29&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O29" s="18"/>
@@ -1813,7 +1808,7 @@
         <v>3</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C30" s="19"/>
       <c r="D30" s="19"/>
@@ -1830,7 +1825,7 @@
       </c>
       <c r="M30" s="18"/>
       <c r="N30" s="18">
-        <f>IF(L30&gt;=75,"A1",IF(L30&gt;=70,"B2",IF(L30&gt;=65,"B3",IF(L30&gt;=60,"C4",IF(L30&gt;=55,"C5",IF(L30&gt;=50,"C6",IF(N30&gt;=45,"D7",IF(L30&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L30&gt;=75,"A1",IF(L30&gt;=70,"B2",IF(L30&gt;=65,"B3",IF(L30&gt;=60,"C4",IF(L30&gt;=55,"C5",IF(L30&gt;=50,"C6",IF(L30&gt;=45,"D7",IF(L30&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O30" s="18"/>
@@ -1856,7 +1851,7 @@
         <v>4</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C31" s="19"/>
       <c r="D31" s="19"/>
@@ -1873,7 +1868,7 @@
       </c>
       <c r="M31" s="18"/>
       <c r="N31" s="18">
-        <f>IF(L31&gt;=75,"A1",IF(L31&gt;=70,"B2",IF(L31&gt;=65,"B3",IF(L31&gt;=60,"C4",IF(L31&gt;=55,"C5",IF(L31&gt;=50,"C6",IF(N31&gt;=45,"D7",IF(L31&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L31&gt;=75,"A1",IF(L31&gt;=70,"B2",IF(L31&gt;=65,"B3",IF(L31&gt;=60,"C4",IF(L31&gt;=55,"C5",IF(L31&gt;=50,"C6",IF(L31&gt;=45,"D7",IF(L31&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O31" s="18"/>
@@ -1899,7 +1894,7 @@
         <v>5</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C32" s="19"/>
       <c r="D32" s="19"/>
@@ -1916,7 +1911,7 @@
       </c>
       <c r="M32" s="18"/>
       <c r="N32" s="18">
-        <f>IF(L32&gt;=75,"A1",IF(L32&gt;=70,"B2",IF(L32&gt;=65,"B3",IF(L32&gt;=60,"C4",IF(L32&gt;=55,"C5",IF(L32&gt;=50,"C6",IF(N32&gt;=45,"D7",IF(L32&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L32&gt;=75,"A1",IF(L32&gt;=70,"B2",IF(L32&gt;=65,"B3",IF(L32&gt;=60,"C4",IF(L32&gt;=55,"C5",IF(L32&gt;=50,"C6",IF(L32&gt;=45,"D7",IF(L32&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O32" s="18"/>
@@ -1942,7 +1937,7 @@
         <v>6</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C33" s="19"/>
       <c r="D33" s="19"/>
@@ -1959,7 +1954,7 @@
       </c>
       <c r="M33" s="18"/>
       <c r="N33" s="18">
-        <f>IF(L33&gt;=75,"A1",IF(L33&gt;=70,"B2",IF(L33&gt;=65,"B3",IF(L33&gt;=60,"C4",IF(L33&gt;=55,"C5",IF(L33&gt;=50,"C6",IF(N33&gt;=45,"D7",IF(L33&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L33&gt;=75,"A1",IF(L33&gt;=70,"B2",IF(L33&gt;=65,"B3",IF(L33&gt;=60,"C4",IF(L33&gt;=55,"C5",IF(L33&gt;=50,"C6",IF(L33&gt;=45,"D7",IF(L33&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O33" s="18"/>
@@ -1985,7 +1980,7 @@
         <v>7</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C34" s="19"/>
       <c r="D34" s="19"/>
@@ -2002,7 +1997,7 @@
       </c>
       <c r="M34" s="18"/>
       <c r="N34" s="18">
-        <f>IF(L34&gt;=75,"A1",IF(L34&gt;=70,"B2",IF(L34&gt;=65,"B3",IF(L34&gt;=60,"C4",IF(L34&gt;=55,"C5",IF(L34&gt;=50,"C6",IF(N34&gt;=45,"D7",IF(L34&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L34&gt;=75,"A1",IF(L34&gt;=70,"B2",IF(L34&gt;=65,"B3",IF(L34&gt;=60,"C4",IF(L34&gt;=55,"C5",IF(L34&gt;=50,"C6",IF(L34&gt;=45,"D7",IF(L34&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O34" s="18"/>
@@ -2028,7 +2023,7 @@
         <v>8</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C35" s="19"/>
       <c r="D35" s="19"/>
@@ -2045,7 +2040,7 @@
       </c>
       <c r="M35" s="18"/>
       <c r="N35" s="18">
-        <f>IF(L35&gt;=75,"A1",IF(L35&gt;=70,"B2",IF(L35&gt;=65,"B3",IF(L35&gt;=60,"C4",IF(L35&gt;=55,"C5",IF(L35&gt;=50,"C6",IF(N35&gt;=45,"D7",IF(L35&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L35&gt;=75,"A1",IF(L35&gt;=70,"B2",IF(L35&gt;=65,"B3",IF(L35&gt;=60,"C4",IF(L35&gt;=55,"C5",IF(L35&gt;=50,"C6",IF(L35&gt;=45,"D7",IF(L35&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O35" s="18"/>
@@ -2071,7 +2066,7 @@
         <v>9</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C36" s="19"/>
       <c r="D36" s="19"/>
@@ -2088,7 +2083,7 @@
       </c>
       <c r="M36" s="18"/>
       <c r="N36" s="18">
-        <f>IF(L36&gt;=75,"A1",IF(L36&gt;=70,"B2",IF(L36&gt;=65,"B3",IF(L36&gt;=60,"C4",IF(L36&gt;=55,"C5",IF(L36&gt;=50,"C6",IF(N36&gt;=45,"D7",IF(L36&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L36&gt;=75,"A1",IF(L36&gt;=70,"B2",IF(L36&gt;=65,"B3",IF(L36&gt;=60,"C4",IF(L36&gt;=55,"C5",IF(L36&gt;=50,"C6",IF(L36&gt;=45,"D7",IF(L36&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O36" s="18"/>
@@ -2110,7 +2105,7 @@
         <v>10</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C37" s="19"/>
       <c r="D37" s="19"/>
@@ -2127,7 +2122,7 @@
       </c>
       <c r="M37" s="18"/>
       <c r="N37" s="18">
-        <f>IF(L37&gt;=75,"A1",IF(L37&gt;=70,"B2",IF(L37&gt;=65,"B3",IF(L37&gt;=60,"C4",IF(L37&gt;=55,"C5",IF(L37&gt;=50,"C6",IF(N37&gt;=45,"D7",IF(L37&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L37&gt;=75,"A1",IF(L37&gt;=70,"B2",IF(L37&gt;=65,"B3",IF(L37&gt;=60,"C4",IF(L37&gt;=55,"C5",IF(L37&gt;=50,"C6",IF(L37&gt;=45,"D7",IF(L37&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O37" s="18"/>
@@ -2140,7 +2135,7 @@
         <v>11</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C38" s="19"/>
       <c r="D38" s="19"/>
@@ -2157,7 +2152,7 @@
       </c>
       <c r="M38" s="18"/>
       <c r="N38" s="18">
-        <f>IF(L38&gt;=75,"A1",IF(L38&gt;=70,"B2",IF(L38&gt;=65,"B3",IF(L38&gt;=60,"C4",IF(L38&gt;=55,"C5",IF(L38&gt;=50,"C6",IF(N38&gt;=45,"D7",IF(L38&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L38&gt;=75,"A1",IF(L38&gt;=70,"B2",IF(L38&gt;=65,"B3",IF(L38&gt;=60,"C4",IF(L38&gt;=55,"C5",IF(L38&gt;=50,"C6",IF(L38&gt;=45,"D7",IF(L38&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O38" s="18"/>
@@ -2179,7 +2174,7 @@
         <v>12</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C39" s="19"/>
       <c r="D39" s="19"/>
@@ -2196,7 +2191,7 @@
       </c>
       <c r="M39" s="18"/>
       <c r="N39" s="18">
-        <f>IF(L39&gt;=75,"A1",IF(L39&gt;=70,"B2",IF(L39&gt;=65,"B3",IF(L39&gt;=60,"C4",IF(L39&gt;=55,"C5",IF(L39&gt;=50,"C6",IF(N39&gt;=45,"D7",IF(L39&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L39&gt;=75,"A1",IF(L39&gt;=70,"B2",IF(L39&gt;=65,"B3",IF(L39&gt;=60,"C4",IF(L39&gt;=55,"C5",IF(L39&gt;=50,"C6",IF(L39&gt;=45,"D7",IF(L39&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O39" s="18"/>
@@ -2218,7 +2213,7 @@
         <v>13</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C40" s="19"/>
       <c r="D40" s="19"/>
@@ -2235,7 +2230,7 @@
       </c>
       <c r="M40" s="18"/>
       <c r="N40" s="18">
-        <f>IF(L40&gt;=75,"A1",IF(L40&gt;=70,"B2",IF(L40&gt;=65,"B3",IF(L40&gt;=60,"C4",IF(L40&gt;=55,"C5",IF(L40&gt;=50,"C6",IF(N40&gt;=45,"D7",IF(L40&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L40&gt;=75,"A1",IF(L40&gt;=70,"B2",IF(L40&gt;=65,"B3",IF(L40&gt;=60,"C4",IF(L40&gt;=55,"C5",IF(L40&gt;=50,"C6",IF(L40&gt;=45,"D7",IF(L40&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O40" s="18"/>
@@ -2257,7 +2252,7 @@
         <v>14</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C41" s="19"/>
       <c r="D41" s="19"/>
@@ -2274,7 +2269,7 @@
       </c>
       <c r="M41" s="18"/>
       <c r="N41" s="18">
-        <f>IF(L41&gt;=75,"A1",IF(L41&gt;=70,"B2",IF(L41&gt;=65,"B3",IF(L41&gt;=60,"C4",IF(L41&gt;=55,"C5",IF(L41&gt;=50,"C6",IF(N41&gt;=45,"D7",IF(L41&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L41&gt;=75,"A1",IF(L41&gt;=70,"B2",IF(L41&gt;=65,"B3",IF(L41&gt;=60,"C4",IF(L41&gt;=55,"C5",IF(L41&gt;=50,"C6",IF(L41&gt;=45,"D7",IF(L41&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O41" s="18"/>
@@ -2296,7 +2291,7 @@
         <v>15</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="19"/>
@@ -2313,7 +2308,7 @@
       </c>
       <c r="M42" s="18"/>
       <c r="N42" s="18">
-        <f>IF(L42&gt;=75,"A1",IF(L42&gt;=70,"B2",IF(L42&gt;=65,"B3",IF(L42&gt;=60,"C4",IF(L42&gt;=55,"C5",IF(L42&gt;=50,"C6",IF(N42&gt;=45,"D7",IF(L42&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L42&gt;=75,"A1",IF(L42&gt;=70,"B2",IF(L42&gt;=65,"B3",IF(L42&gt;=60,"C4",IF(L42&gt;=55,"C5",IF(L42&gt;=50,"C6",IF(L42&gt;=45,"D7",IF(L42&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O42" s="18"/>
@@ -2331,22 +2326,30 @@
       <c r="Z42" s="14"/>
     </row>
     <row r="43" spans="1:26">
-      <c r="A43" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20"/>
+      <c r="A43" s="18">
+        <v>16</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C43" s="19"/>
+      <c r="D43" s="19"/>
+      <c r="E43" s="19"/>
+      <c r="F43" s="19"/>
       <c r="G43" s="18"/>
       <c r="H43" s="18"/>
       <c r="I43" s="18"/>
       <c r="J43" s="18"/>
       <c r="K43" s="18"/>
-      <c r="L43" s="18"/>
+      <c r="L43" s="18">
+        <f>SUM(G43, H43, J43)</f>
+        <v>0</v>
+      </c>
       <c r="M43" s="18"/>
-      <c r="N43" s="18"/>
+      <c r="N43" s="18">
+        <f>IF(L43&gt;=75,"A1",IF(L43&gt;=70,"B2",IF(L43&gt;=65,"B3",IF(L43&gt;=60,"C4",IF(L43&gt;=55,"C5",IF(L43&gt;=50,"C6",IF(L43&gt;=45,"D7",IF(L43&gt;=40,"E8","F9"))))))))</f>
+        <v>0</v>
+      </c>
       <c r="O43" s="18"/>
       <c r="P43" s="18"/>
       <c r="Q43" s="18"/>
@@ -2363,7 +2366,7 @@
     </row>
     <row r="44" spans="1:26">
       <c r="A44" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B44" s="20"/>
       <c r="C44" s="20"/>
@@ -2394,7 +2397,7 @@
     </row>
     <row r="45" spans="1:26">
       <c r="A45" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B45" s="20"/>
       <c r="C45" s="20"/>
@@ -2425,7 +2428,7 @@
     </row>
     <row r="46" spans="1:26">
       <c r="A46" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B46" s="20"/>
       <c r="C46" s="20"/>
@@ -2456,7 +2459,7 @@
     </row>
     <row r="47" spans="1:26">
       <c r="A47" s="20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B47" s="20"/>
       <c r="C47" s="20"/>
@@ -2478,7 +2481,7 @@
     </row>
     <row r="48" spans="1:26">
       <c r="A48" s="20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B48" s="20"/>
       <c r="C48" s="20"/>
@@ -2508,7 +2511,7 @@
     </row>
     <row r="49" spans="1:26">
       <c r="A49" s="20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B49" s="20"/>
       <c r="C49" s="20"/>
@@ -2538,7 +2541,7 @@
     </row>
     <row r="50" spans="1:26">
       <c r="A50" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B50" s="20"/>
       <c r="C50" s="20"/>
@@ -2567,6 +2570,26 @@
       <c r="Y50" s="15"/>
     </row>
     <row r="51" spans="1:26">
+      <c r="A51" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B51" s="20"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18"/>
+      <c r="I51" s="18"/>
+      <c r="J51" s="18"/>
+      <c r="K51" s="18"/>
+      <c r="L51" s="18"/>
+      <c r="M51" s="18"/>
+      <c r="N51" s="18"/>
+      <c r="O51" s="18"/>
+      <c r="P51" s="18"/>
+      <c r="Q51" s="18"/>
+      <c r="R51" s="18"/>
       <c r="T51" s="13" t="s">
         <v>109</v>
       </c>
@@ -2610,7 +2633,7 @@
     </row>
     <row r="59" spans="1:26">
       <c r="A59" s="17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B59" s="17" t="s">
         <v>111</v>
@@ -2626,7 +2649,7 @@
       </c>
       <c r="H59" s="17"/>
       <c r="J59" s="17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K59" s="17" t="s">
         <v>122</v>
@@ -3057,7 +3080,7 @@
       <c r="Z78" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="254">
+  <mergeCells count="260">
     <mergeCell ref="F1:U2"/>
     <mergeCell ref="F3:U4"/>
     <mergeCell ref="F5:U5"/>
@@ -3195,8 +3218,12 @@
     <mergeCell ref="L42:M42"/>
     <mergeCell ref="N42:O42"/>
     <mergeCell ref="P42:R42"/>
-    <mergeCell ref="A43:F43"/>
-    <mergeCell ref="G43:R43"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="N43:O43"/>
+    <mergeCell ref="P43:R43"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="G44:R44"/>
     <mergeCell ref="A45:F45"/>
@@ -3211,6 +3238,8 @@
     <mergeCell ref="G49:R49"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="G50:R50"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="G51:R51"/>
     <mergeCell ref="T24:Z24"/>
     <mergeCell ref="U25:V25"/>
     <mergeCell ref="W25:Z25"/>

</xml_diff>

<commit_message>
Fix all SS2 scores with user-provided data, remove Balogun overrides
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Hiktaos_Primary_Final.xlsx
+++ b/Hiktaos_Primary_Final.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="145">
   <si>
     <t>HIKTAOS</t>
   </si>
@@ -116,9 +116,6 @@
     <t>Attendance Percentage</t>
   </si>
   <si>
-    <t>%</t>
-  </si>
-  <si>
     <t>ACADEMIC PERFORMANCE</t>
   </si>
   <si>
@@ -153,49 +150,52 @@
 IN SUBJECT</t>
   </si>
   <si>
-    <t>English Studies</t>
+    <t>Social Studies</t>
+  </si>
+  <si>
+    <t>Civic Education</t>
+  </si>
+  <si>
+    <t>CRS</t>
+  </si>
+  <si>
+    <t>Security Education</t>
+  </si>
+  <si>
+    <t>History</t>
+  </si>
+  <si>
+    <t>Agricultural Science</t>
+  </si>
+  <si>
+    <t>Home Economics</t>
+  </si>
+  <si>
+    <t>Basic Science</t>
+  </si>
+  <si>
+    <t>PHE</t>
+  </si>
+  <si>
+    <t>ICT</t>
+  </si>
+  <si>
+    <t>Cultural &amp; Creative Arts</t>
   </si>
   <si>
     <t>Mathematics</t>
   </si>
   <si>
-    <t>Basic Science &amp; Tech</t>
-  </si>
-  <si>
-    <t>Social Studies</t>
-  </si>
-  <si>
-    <t>Civic Education</t>
-  </si>
-  <si>
-    <t>Cultural &amp; Creative Arts</t>
-  </si>
-  <si>
-    <t>Physical &amp; Health Education</t>
-  </si>
-  <si>
-    <t>Agricultural Science</t>
-  </si>
-  <si>
-    <t>Home Economics</t>
-  </si>
-  <si>
-    <t>CRS / IRS</t>
-  </si>
-  <si>
-    <t>Yoruba Language</t>
+    <t>English Language</t>
+  </si>
+  <si>
+    <t>Verbal Reasoning</t>
   </si>
   <si>
     <t>Quantitative Reasoning</t>
   </si>
   <si>
-    <t>Verbal Reasoning</t>
-  </si>
-  <si>
-    <t>Handwriting</t>
-  </si>
-  <si>
-    <t>French</t>
+    <t>Vocational Studies</t>
   </si>
   <si>
     <t>TOTAL MARKS</t>
@@ -759,8 +759,8 @@
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>136398</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>12573</xdr:rowOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>136398</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1081,7 +1081,7 @@
     <col min="1" max="26" width="4.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="40" customHeight="1">
+    <row r="1" spans="1:26">
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1446,9 +1446,7 @@
       <c r="J17" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="M17" s="13" t="s">
-        <v>9</v>
-      </c>
+      <c r="M17" s="14"/>
       <c r="N17" s="14"/>
       <c r="O17" s="14"/>
       <c r="P17" s="14"/>
@@ -1550,9 +1548,6 @@
       <c r="W20" s="13"/>
       <c r="X20" s="15"/>
       <c r="Y20" s="15"/>
-      <c r="Z20" s="13" t="s">
-        <v>33</v>
-      </c>
     </row>
     <row r="21" spans="1:26">
       <c r="A21" s="13" t="s">
@@ -1607,7 +1602,7 @@
     </row>
     <row r="24" spans="1:26">
       <c r="A24" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -1638,34 +1633,34 @@
     </row>
     <row r="25" spans="1:26">
       <c r="A25" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="B25" s="16" t="s">
-        <v>36</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
       <c r="G25" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K25" s="16"/>
       <c r="L25" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="M25" s="16"/>
       <c r="N25" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O25" s="16"/>
       <c r="P25" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q25" s="16"/>
       <c r="R25" s="16"/>
@@ -1673,7 +1668,7 @@
         <v>68</v>
       </c>
       <c r="U25" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="V25" s="17"/>
       <c r="W25" s="17" t="s">
@@ -1691,10 +1686,10 @@
       <c r="E26" s="16"/>
       <c r="F26" s="16"/>
       <c r="G26" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H26" s="16" t="s">
         <v>38</v>
-      </c>
-      <c r="H26" s="16" t="s">
-        <v>39</v>
       </c>
       <c r="I26" s="16"/>
       <c r="J26" s="16"/>
@@ -1727,7 +1722,7 @@
         <v>1</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="19"/>
@@ -1744,7 +1739,7 @@
       </c>
       <c r="M28" s="18"/>
       <c r="N28" s="18">
-        <f>IF(L28&gt;=75,"A1",IF(L28&gt;=70,"B2",IF(L28&gt;=65,"B3",IF(L28&gt;=60,"C4",IF(L28&gt;=55,"C5",IF(L28&gt;=50,"C6",IF(N28&gt;=45,"D7",IF(L28&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L28&gt;=75,"A1",IF(L28&gt;=70,"B2",IF(L28&gt;=65,"B3",IF(L28&gt;=60,"C4",IF(L28&gt;=55,"C5",IF(L28&gt;=50,"C6",IF(L28&gt;=45,"D7",IF(L28&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O28" s="18"/>
@@ -1770,7 +1765,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="19"/>
@@ -1787,7 +1782,7 @@
       </c>
       <c r="M29" s="18"/>
       <c r="N29" s="18">
-        <f>IF(L29&gt;=75,"A1",IF(L29&gt;=70,"B2",IF(L29&gt;=65,"B3",IF(L29&gt;=60,"C4",IF(L29&gt;=55,"C5",IF(L29&gt;=50,"C6",IF(N29&gt;=45,"D7",IF(L29&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L29&gt;=75,"A1",IF(L29&gt;=70,"B2",IF(L29&gt;=65,"B3",IF(L29&gt;=60,"C4",IF(L29&gt;=55,"C5",IF(L29&gt;=50,"C6",IF(L29&gt;=45,"D7",IF(L29&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O29" s="18"/>
@@ -1813,7 +1808,7 @@
         <v>3</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C30" s="19"/>
       <c r="D30" s="19"/>
@@ -1830,7 +1825,7 @@
       </c>
       <c r="M30" s="18"/>
       <c r="N30" s="18">
-        <f>IF(L30&gt;=75,"A1",IF(L30&gt;=70,"B2",IF(L30&gt;=65,"B3",IF(L30&gt;=60,"C4",IF(L30&gt;=55,"C5",IF(L30&gt;=50,"C6",IF(N30&gt;=45,"D7",IF(L30&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L30&gt;=75,"A1",IF(L30&gt;=70,"B2",IF(L30&gt;=65,"B3",IF(L30&gt;=60,"C4",IF(L30&gt;=55,"C5",IF(L30&gt;=50,"C6",IF(L30&gt;=45,"D7",IF(L30&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O30" s="18"/>
@@ -1856,7 +1851,7 @@
         <v>4</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C31" s="19"/>
       <c r="D31" s="19"/>
@@ -1873,7 +1868,7 @@
       </c>
       <c r="M31" s="18"/>
       <c r="N31" s="18">
-        <f>IF(L31&gt;=75,"A1",IF(L31&gt;=70,"B2",IF(L31&gt;=65,"B3",IF(L31&gt;=60,"C4",IF(L31&gt;=55,"C5",IF(L31&gt;=50,"C6",IF(N31&gt;=45,"D7",IF(L31&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L31&gt;=75,"A1",IF(L31&gt;=70,"B2",IF(L31&gt;=65,"B3",IF(L31&gt;=60,"C4",IF(L31&gt;=55,"C5",IF(L31&gt;=50,"C6",IF(L31&gt;=45,"D7",IF(L31&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O31" s="18"/>
@@ -1899,7 +1894,7 @@
         <v>5</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C32" s="19"/>
       <c r="D32" s="19"/>
@@ -1916,7 +1911,7 @@
       </c>
       <c r="M32" s="18"/>
       <c r="N32" s="18">
-        <f>IF(L32&gt;=75,"A1",IF(L32&gt;=70,"B2",IF(L32&gt;=65,"B3",IF(L32&gt;=60,"C4",IF(L32&gt;=55,"C5",IF(L32&gt;=50,"C6",IF(N32&gt;=45,"D7",IF(L32&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L32&gt;=75,"A1",IF(L32&gt;=70,"B2",IF(L32&gt;=65,"B3",IF(L32&gt;=60,"C4",IF(L32&gt;=55,"C5",IF(L32&gt;=50,"C6",IF(L32&gt;=45,"D7",IF(L32&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O32" s="18"/>
@@ -1942,7 +1937,7 @@
         <v>6</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C33" s="19"/>
       <c r="D33" s="19"/>
@@ -1959,7 +1954,7 @@
       </c>
       <c r="M33" s="18"/>
       <c r="N33" s="18">
-        <f>IF(L33&gt;=75,"A1",IF(L33&gt;=70,"B2",IF(L33&gt;=65,"B3",IF(L33&gt;=60,"C4",IF(L33&gt;=55,"C5",IF(L33&gt;=50,"C6",IF(N33&gt;=45,"D7",IF(L33&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L33&gt;=75,"A1",IF(L33&gt;=70,"B2",IF(L33&gt;=65,"B3",IF(L33&gt;=60,"C4",IF(L33&gt;=55,"C5",IF(L33&gt;=50,"C6",IF(L33&gt;=45,"D7",IF(L33&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O33" s="18"/>
@@ -1985,7 +1980,7 @@
         <v>7</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C34" s="19"/>
       <c r="D34" s="19"/>
@@ -2002,7 +1997,7 @@
       </c>
       <c r="M34" s="18"/>
       <c r="N34" s="18">
-        <f>IF(L34&gt;=75,"A1",IF(L34&gt;=70,"B2",IF(L34&gt;=65,"B3",IF(L34&gt;=60,"C4",IF(L34&gt;=55,"C5",IF(L34&gt;=50,"C6",IF(N34&gt;=45,"D7",IF(L34&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L34&gt;=75,"A1",IF(L34&gt;=70,"B2",IF(L34&gt;=65,"B3",IF(L34&gt;=60,"C4",IF(L34&gt;=55,"C5",IF(L34&gt;=50,"C6",IF(L34&gt;=45,"D7",IF(L34&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O34" s="18"/>
@@ -2028,7 +2023,7 @@
         <v>8</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C35" s="19"/>
       <c r="D35" s="19"/>
@@ -2045,7 +2040,7 @@
       </c>
       <c r="M35" s="18"/>
       <c r="N35" s="18">
-        <f>IF(L35&gt;=75,"A1",IF(L35&gt;=70,"B2",IF(L35&gt;=65,"B3",IF(L35&gt;=60,"C4",IF(L35&gt;=55,"C5",IF(L35&gt;=50,"C6",IF(N35&gt;=45,"D7",IF(L35&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L35&gt;=75,"A1",IF(L35&gt;=70,"B2",IF(L35&gt;=65,"B3",IF(L35&gt;=60,"C4",IF(L35&gt;=55,"C5",IF(L35&gt;=50,"C6",IF(L35&gt;=45,"D7",IF(L35&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O35" s="18"/>
@@ -2071,7 +2066,7 @@
         <v>9</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C36" s="19"/>
       <c r="D36" s="19"/>
@@ -2088,7 +2083,7 @@
       </c>
       <c r="M36" s="18"/>
       <c r="N36" s="18">
-        <f>IF(L36&gt;=75,"A1",IF(L36&gt;=70,"B2",IF(L36&gt;=65,"B3",IF(L36&gt;=60,"C4",IF(L36&gt;=55,"C5",IF(L36&gt;=50,"C6",IF(N36&gt;=45,"D7",IF(L36&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L36&gt;=75,"A1",IF(L36&gt;=70,"B2",IF(L36&gt;=65,"B3",IF(L36&gt;=60,"C4",IF(L36&gt;=55,"C5",IF(L36&gt;=50,"C6",IF(L36&gt;=45,"D7",IF(L36&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O36" s="18"/>
@@ -2110,7 +2105,7 @@
         <v>10</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C37" s="19"/>
       <c r="D37" s="19"/>
@@ -2127,7 +2122,7 @@
       </c>
       <c r="M37" s="18"/>
       <c r="N37" s="18">
-        <f>IF(L37&gt;=75,"A1",IF(L37&gt;=70,"B2",IF(L37&gt;=65,"B3",IF(L37&gt;=60,"C4",IF(L37&gt;=55,"C5",IF(L37&gt;=50,"C6",IF(N37&gt;=45,"D7",IF(L37&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L37&gt;=75,"A1",IF(L37&gt;=70,"B2",IF(L37&gt;=65,"B3",IF(L37&gt;=60,"C4",IF(L37&gt;=55,"C5",IF(L37&gt;=50,"C6",IF(L37&gt;=45,"D7",IF(L37&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O37" s="18"/>
@@ -2140,7 +2135,7 @@
         <v>11</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C38" s="19"/>
       <c r="D38" s="19"/>
@@ -2157,7 +2152,7 @@
       </c>
       <c r="M38" s="18"/>
       <c r="N38" s="18">
-        <f>IF(L38&gt;=75,"A1",IF(L38&gt;=70,"B2",IF(L38&gt;=65,"B3",IF(L38&gt;=60,"C4",IF(L38&gt;=55,"C5",IF(L38&gt;=50,"C6",IF(N38&gt;=45,"D7",IF(L38&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L38&gt;=75,"A1",IF(L38&gt;=70,"B2",IF(L38&gt;=65,"B3",IF(L38&gt;=60,"C4",IF(L38&gt;=55,"C5",IF(L38&gt;=50,"C6",IF(L38&gt;=45,"D7",IF(L38&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O38" s="18"/>
@@ -2179,7 +2174,7 @@
         <v>12</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C39" s="19"/>
       <c r="D39" s="19"/>
@@ -2196,7 +2191,7 @@
       </c>
       <c r="M39" s="18"/>
       <c r="N39" s="18">
-        <f>IF(L39&gt;=75,"A1",IF(L39&gt;=70,"B2",IF(L39&gt;=65,"B3",IF(L39&gt;=60,"C4",IF(L39&gt;=55,"C5",IF(L39&gt;=50,"C6",IF(N39&gt;=45,"D7",IF(L39&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L39&gt;=75,"A1",IF(L39&gt;=70,"B2",IF(L39&gt;=65,"B3",IF(L39&gt;=60,"C4",IF(L39&gt;=55,"C5",IF(L39&gt;=50,"C6",IF(L39&gt;=45,"D7",IF(L39&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O39" s="18"/>
@@ -2218,7 +2213,7 @@
         <v>13</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C40" s="19"/>
       <c r="D40" s="19"/>
@@ -2235,7 +2230,7 @@
       </c>
       <c r="M40" s="18"/>
       <c r="N40" s="18">
-        <f>IF(L40&gt;=75,"A1",IF(L40&gt;=70,"B2",IF(L40&gt;=65,"B3",IF(L40&gt;=60,"C4",IF(L40&gt;=55,"C5",IF(L40&gt;=50,"C6",IF(N40&gt;=45,"D7",IF(L40&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L40&gt;=75,"A1",IF(L40&gt;=70,"B2",IF(L40&gt;=65,"B3",IF(L40&gt;=60,"C4",IF(L40&gt;=55,"C5",IF(L40&gt;=50,"C6",IF(L40&gt;=45,"D7",IF(L40&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O40" s="18"/>
@@ -2257,7 +2252,7 @@
         <v>14</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C41" s="19"/>
       <c r="D41" s="19"/>
@@ -2274,7 +2269,7 @@
       </c>
       <c r="M41" s="18"/>
       <c r="N41" s="18">
-        <f>IF(L41&gt;=75,"A1",IF(L41&gt;=70,"B2",IF(L41&gt;=65,"B3",IF(L41&gt;=60,"C4",IF(L41&gt;=55,"C5",IF(L41&gt;=50,"C6",IF(N41&gt;=45,"D7",IF(L41&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L41&gt;=75,"A1",IF(L41&gt;=70,"B2",IF(L41&gt;=65,"B3",IF(L41&gt;=60,"C4",IF(L41&gt;=55,"C5",IF(L41&gt;=50,"C6",IF(L41&gt;=45,"D7",IF(L41&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O41" s="18"/>
@@ -2296,7 +2291,7 @@
         <v>15</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="19"/>
@@ -2313,7 +2308,7 @@
       </c>
       <c r="M42" s="18"/>
       <c r="N42" s="18">
-        <f>IF(L42&gt;=75,"A1",IF(L42&gt;=70,"B2",IF(L42&gt;=65,"B3",IF(L42&gt;=60,"C4",IF(L42&gt;=55,"C5",IF(L42&gt;=50,"C6",IF(N42&gt;=45,"D7",IF(L42&gt;=40,"E8","F9"))))))))</f>
+        <f>IF(L42&gt;=75,"A1",IF(L42&gt;=70,"B2",IF(L42&gt;=65,"B3",IF(L42&gt;=60,"C4",IF(L42&gt;=55,"C5",IF(L42&gt;=50,"C6",IF(L42&gt;=45,"D7",IF(L42&gt;=40,"E8","F9"))))))))</f>
         <v>0</v>
       </c>
       <c r="O42" s="18"/>
@@ -2331,22 +2326,30 @@
       <c r="Z42" s="14"/>
     </row>
     <row r="43" spans="1:26">
-      <c r="A43" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20"/>
+      <c r="A43" s="18">
+        <v>16</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C43" s="19"/>
+      <c r="D43" s="19"/>
+      <c r="E43" s="19"/>
+      <c r="F43" s="19"/>
       <c r="G43" s="18"/>
       <c r="H43" s="18"/>
       <c r="I43" s="18"/>
       <c r="J43" s="18"/>
       <c r="K43" s="18"/>
-      <c r="L43" s="18"/>
+      <c r="L43" s="18">
+        <f>SUM(G43, H43, J43)</f>
+        <v>0</v>
+      </c>
       <c r="M43" s="18"/>
-      <c r="N43" s="18"/>
+      <c r="N43" s="18">
+        <f>IF(L43&gt;=75,"A1",IF(L43&gt;=70,"B2",IF(L43&gt;=65,"B3",IF(L43&gt;=60,"C4",IF(L43&gt;=55,"C5",IF(L43&gt;=50,"C6",IF(L43&gt;=45,"D7",IF(L43&gt;=40,"E8","F9"))))))))</f>
+        <v>0</v>
+      </c>
       <c r="O43" s="18"/>
       <c r="P43" s="18"/>
       <c r="Q43" s="18"/>
@@ -2363,7 +2366,7 @@
     </row>
     <row r="44" spans="1:26">
       <c r="A44" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B44" s="20"/>
       <c r="C44" s="20"/>
@@ -2394,7 +2397,7 @@
     </row>
     <row r="45" spans="1:26">
       <c r="A45" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B45" s="20"/>
       <c r="C45" s="20"/>
@@ -2425,7 +2428,7 @@
     </row>
     <row r="46" spans="1:26">
       <c r="A46" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B46" s="20"/>
       <c r="C46" s="20"/>
@@ -2456,7 +2459,7 @@
     </row>
     <row r="47" spans="1:26">
       <c r="A47" s="20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B47" s="20"/>
       <c r="C47" s="20"/>
@@ -2478,7 +2481,7 @@
     </row>
     <row r="48" spans="1:26">
       <c r="A48" s="20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B48" s="20"/>
       <c r="C48" s="20"/>
@@ -2508,7 +2511,7 @@
     </row>
     <row r="49" spans="1:26">
       <c r="A49" s="20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B49" s="20"/>
       <c r="C49" s="20"/>
@@ -2538,7 +2541,7 @@
     </row>
     <row r="50" spans="1:26">
       <c r="A50" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B50" s="20"/>
       <c r="C50" s="20"/>
@@ -2567,6 +2570,26 @@
       <c r="Y50" s="15"/>
     </row>
     <row r="51" spans="1:26">
+      <c r="A51" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B51" s="20"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18"/>
+      <c r="I51" s="18"/>
+      <c r="J51" s="18"/>
+      <c r="K51" s="18"/>
+      <c r="L51" s="18"/>
+      <c r="M51" s="18"/>
+      <c r="N51" s="18"/>
+      <c r="O51" s="18"/>
+      <c r="P51" s="18"/>
+      <c r="Q51" s="18"/>
+      <c r="R51" s="18"/>
       <c r="T51" s="13" t="s">
         <v>109</v>
       </c>
@@ -2610,7 +2633,7 @@
     </row>
     <row r="59" spans="1:26">
       <c r="A59" s="17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B59" s="17" t="s">
         <v>111</v>
@@ -2626,7 +2649,7 @@
       </c>
       <c r="H59" s="17"/>
       <c r="J59" s="17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K59" s="17" t="s">
         <v>122</v>
@@ -3057,7 +3080,7 @@
       <c r="Z78" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="254">
+  <mergeCells count="260">
     <mergeCell ref="F1:U2"/>
     <mergeCell ref="F3:U4"/>
     <mergeCell ref="F5:U5"/>
@@ -3195,8 +3218,12 @@
     <mergeCell ref="L42:M42"/>
     <mergeCell ref="N42:O42"/>
     <mergeCell ref="P42:R42"/>
-    <mergeCell ref="A43:F43"/>
-    <mergeCell ref="G43:R43"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="N43:O43"/>
+    <mergeCell ref="P43:R43"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="G44:R44"/>
     <mergeCell ref="A45:F45"/>
@@ -3211,6 +3238,8 @@
     <mergeCell ref="G49:R49"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="G50:R50"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="G51:R51"/>
     <mergeCell ref="T24:Z24"/>
     <mergeCell ref="U25:V25"/>
     <mergeCell ref="W25:Z25"/>

</xml_diff>